<commit_message>
EAN för nya skal, vit Lightning-kabel borttagen
Skal till iPhone 17, 17 Pro och 18 Pro har EAN i produktdatan.
Den vita USB-C till Lightning-kabeln säljs inte och är borttagen ur
produktdata, bildpaket, startsidan och filmen (ersatt av svart
iPhone 17-skal i montaget). FAQ om EAN uppdaterad.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/aterforsaljare/corder-produktdata.xlsx
+++ b/docs/aterforsaljare/corder-produktdata.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1681,7 +1681,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>7350140690788</t>
+        </is>
+      </c>
       <c r="G30" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17-black.webp</t>
@@ -1719,7 +1723,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>7350140690795</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17-skogsgron.webp</t>
@@ -1757,7 +1765,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>7350140690801</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17p-black.webp</t>
@@ -1795,7 +1807,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>7350140690818</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17p-skogsgron.webp</t>
@@ -1833,7 +1849,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>7350140690825</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17p-black.webp</t>
@@ -1871,7 +1891,11 @@
           <t>TPU, matt</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>7350140690832</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>https://corder.se/img/cut/17p-skogsgron.webp</t>
@@ -1988,7 +2012,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Laddkabel USB-C till Lightning, 2 m, flätad, vit</t>
+          <t>Laddkabel USB-A till Lightning, 2 m, flätad</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2000,13 +2024,17 @@
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>USB-C / Lightning</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
+          <t>USB-A / Lightning</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>7350140690030</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://corder.se/img/produkter/kabel-usb-c-lightning-vit.webp</t>
+          <t>https://corder.se/img/produkter/kabel-usb-a-lightning-2m.webp</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2018,29 +2046,29 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Laddkabel USB-A till Lightning, 2 m, flätad</t>
+          <t>Snabbladdare 20W USB-C</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Laddkabel</t>
+          <t>Snabbladdare</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>USB-A / Lightning</t>
+          <t>USB-C, 20 W</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>7350140690030</t>
+          <t>7350140690504</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://corder.se/img/produkter/kabel-usb-a-lightning-2m.webp</t>
+          <t>https://corder.se/img/produkter/laddare-20w-usb-c.webp</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2052,7 +2080,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Snabbladdare 20W USB-C</t>
+          <t>Snabbladdare 20W Dual Port</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2064,17 +2092,17 @@
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>USB-C, 20 W</t>
+          <t>USB-C + USB-A, 20 W</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>7350140690504</t>
+          <t>7350140690771</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://corder.se/img/produkter/laddare-20w-usb-c.webp</t>
+          <t>https://corder.se/img/produkter/laddare-20w-dual-port.webp</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2086,7 +2114,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Snabbladdare 20W Dual Port</t>
+          <t>Snabbladdare 18W USB-A</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2098,54 +2126,20 @@
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>USB-C + USB-A, 20 W</t>
+          <t>USB-A, 18 W, QC 3.0</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>7350140690771</t>
+          <t>7350140690078</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://corder.se/img/produkter/laddare-20w-dual-port.webp</t>
+          <t>https://corder.se/img/produkter/laddare-18w-usb-a.webp</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
-        <is>
-          <t>https://corder.se/#laddning</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Snabbladdare 18W USB-A</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Snabbladdare</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>USB-A, 18 W, QC 3.0</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>7350140690078</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>https://corder.se/img/produkter/laddare-18w-usb-a.webp</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
         <is>
           <t>https://corder.se/#laddning</t>
         </is>

</xml_diff>